<commit_message>
Update score calculation: treat missing parameters as 0 score & restore 21 parameters
</commit_message>
<xml_diff>
--- a/data/weeks/ANM_PS_04_06_2026-10_06_2026.xlsx
+++ b/data/weeks/ANM_PS_04_06_2026-10_06_2026.xlsx
@@ -535,67 +535,67 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="F2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="G2" t="n">
-        <v>0.04</v>
+        <v>0.025</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="I2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="J2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="K2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="L2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="M2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="O2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="P2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="R2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="S2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="T2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="U2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="3">

</xml_diff>